<commit_message>
Ancla del Alma: el agua del atardecer (W1) en el manual, el 3D y la lista de materiales
Panel DTF con transparencia sobre raso esmeralda, del horizonte al galón.
Manual de 33 páginas con la sección 10.1, P13 en el despiece y el plan de corte,
peso ≈ 2,4 kg y ≈ 262 horas-persona.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/materiales/lista-de-materiales.xlsx
+++ b/materiales/lista-de-materiales.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="L6" s="14" t="inlineStr">
         <is>
-          <t>27 oct (F05)</t>
+          <t>26 oct (F04)</t>
         </is>
       </c>
       <c r="M6" s="15" t="inlineStr">
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="E7" s="16" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
@@ -1043,12 +1043,12 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>Forro: entero con tela de 1,50 m; con 1,40 m, dos mitades encontradas en el mismo largo</t>
+          <t>Forro: entero con tela de 1,50 m; con 1,40 m, dos mitades encontradas en el mismo largo (2,3 m). Panel del agua: 0,6 m (pieza de 137 × 56 cm al través)</t>
         </is>
       </c>
       <c r="J7" s="15" t="inlineStr">
         <is>
-          <t>3 Forro</t>
+          <t>3 Forro, 6 Cuerpo de terciopelo</t>
         </is>
       </c>
       <c r="K7" s="14" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>11 nov (F17)</t>
+          <t>26 oct (F04)</t>
         </is>
       </c>
       <c r="M7" s="15" t="inlineStr">
@@ -1218,11 +1218,11 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Pliego de 56 × 98 cm (película de 60 cm), PNG a 300 ppp, polvo antimigración, capa blanca al 50 %</t>
+          <t>Pliego de piezas de 56 × 98 cm a 300 ppp y pliego del agua de 56 × 133,5 cm a 150 ppp con transparencia (medios tonos); película de 60 cm, polvo antimigración, capa blanca al 50 %</t>
         </is>
       </c>
       <c r="E10" s="22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
@@ -1238,12 +1238,12 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>Uno de producción y una tira de prueba (prueba 2)</t>
+          <t>Pliego de piezas y pliego del agua, cada uno con su tira de prueba (prueba 2)</t>
         </is>
       </c>
       <c r="J10" s="15" t="inlineStr">
         <is>
-          <t>8 Apliques: cruz y paneles DTF</t>
+          <t>6 Cuerpo de terciopelo, 8 Apliques: cruz y paneles DTF</t>
         </is>
       </c>
       <c r="K10" s="14" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="M10" s="15" t="inlineStr">
         <is>
-          <t>La tira de prueba ya. El pliego de producción solo después de medir la réplica y aprobar la prueba 2.</t>
+          <t>Las dos tiras de prueba ya (piezas y agua). Los pliegos de producción solo después de medir la réplica y aprobar la prueba 2.</t>
         </is>
       </c>
       <c r="N10" s="19" t="n"/>
@@ -5355,7 +5355,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Peso estimado 1,9–2,7 kg. El peso admisible de la réplica está PENDIENTE (prueba 6).</t>
+          <t>Peso estimado 2,0–2,8 kg. El peso admisible de la réplica está PENDIENTE (prueba 6).</t>
         </is>
       </c>
     </row>
@@ -5577,21 +5577,21 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Terciopelo esmeralda profundo de un solo tono, con el pelo hacia arriba. Trapecio de 67,5 cm arriba, 150 cm al pie y 200 cm de alto. Si la tela no da el ancho del pie, dos nesgas que quedan bajo el galón.</t>
+          <t>Terciopelo esmeralda profundo de un solo tono, con el pelo hacia arriba. Trapecio de 67,5 cm arriba, 150 cm al pie y 200 cm de alto. Si la tela no da el ancho del pie, dos nesgas que quedan bajo el galón. Del horizonte al galón lleva aplicado el panel del agua: raso esmeralda hondo con el DTF del atardecer (W1), con los bordes doblados bajo el cordón del horizonte y bajo el galón.</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>M01</t>
+          <t>M01, M02, M05</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>F04, F05</t>
         </is>
       </c>
       <c r="G10" s="22" t="n">
-        <v>790</v>
+        <v>880</v>
       </c>
     </row>
     <row r="11">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>Sube desde la orla del pie y se aclara en cinco tramos: Capri y aguamarina abajo, cristal en medio, champán y perla arriba. Ninguna piedra toca la película DTF ni se acerca a menos de 4 cm de la amarra o del sol.</t>
+          <t>Sube desde la orla del pie y se aclara en cinco tramos: Capri y aguamarina abajo, cristal en medio, champán y perla arriba. Ninguna piedra va sobre las piezas DTF (azucenas, hojas, olivo, crestas). En el panel del agua se cosen a través de la película, nunca se pegan; bajo el pavé la película ya es casi transparente. Ninguna se acerca a menos de 4 cm de la amarra o del sol.</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
@@ -5813,7 +5813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6295,6 +6295,41 @@
       <c r="G16" s="15" t="inlineStr">
         <is>
           <t>PENDIENTE: puntos de anclaje en el retablo y las andas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="32" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Panel del agua</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>Rectángulo de 137 × 56 cm para prensar; después, trapecio impreso de 111,6 cm arriba, 133,5 cm abajo y 53,3 cm de alto</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>6 mm por los cuatro lados, doblados hacia atrás</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>Se prensa el pliego del agua sobre el raso estirado y se recorta después del reposo. El doblez de arriba queda bajo el cordón del horizonte (y = 140); los de los lados y el pie, 3 mm bajo el borde interior del galón.</t>
         </is>
       </c>
     </row>

</xml_diff>